<commit_message>
auto update queens news 2026-09-28T19:39:21Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Walton Realty NY files plans for 94 units in LIC, partnered with CW Realty as ground lease tenant</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/walton-realty-ny-files-plans-for-94-units-in-lic-cw-realty-signed-ground-lease/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Walton Realty NY submitted a new building construction project for a 94-unit, 86,518-square-foot residential (R-2)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 21-02 44th Drive (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>State advances Astoria project with 139k sf community center, 235 affordable units, school</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/state-advances-astoria-project-with-139k-community-center-235-affordable-units-school/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The nonprofit Variety Boys &amp; Girls Club of Queens secured approval on Friday from the</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development 21-12 30th Road axonometric diagram (Credit - Anthony Shitemi architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-29T18:03:34Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Walton Realty NY files plans for 94 units in LIC, partnered with CW Realty as ground lease tenant</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/walton-realty-ny-files-plans-for-94-units-in-lic-cw-realty-signed-ground-lease/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Walton Realty NY submitted a new building construction project for a 94-unit, 86,518-square-foot residential (R-2)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 21-02 44th Drive (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>State advances Astoria project with 139k sf community center, 235 affordable units, school</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/state-advances-astoria-project-with-139k-community-center-235-affordable-units-school/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>The nonprofit Variety Boys &amp; Girls Club of Queens secured approval on Friday from the</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development 21-12 30th Road axonometric diagram (Credit - Anthony Shitemi architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-09-30T17:59:23Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CDK Capital, Daryl Hagler pay $75.8M for mid-construction project in Ridgewood, sign $10.2M ground lease</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/cdk-capital-darryl-hagler-pay-75-8m-for-mid-construction-project-in-ridgewood-sign-10-2m-ground-lease/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CDK Capital and Daryl Hagler through the entity CDK 3-50 St. Nicholas LLC paid $75.8</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Chart_Frontpage Transfers 3-50 St. Nicholas Avenue (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-01T18:24:06Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CDK Capital, Daryl Hagler pay $75.8M for mid-construction project in Ridgewood, sign $10.2M ground lease</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/cdk-capital-darryl-hagler-pay-75-8m-for-mid-construction-project-in-ridgewood-sign-10-2m-ground-lease/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CDK Capital and Daryl Hagler through the entity CDK 3-50 St. Nicholas LLC paid $75.8</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Chart_Frontpage Transfers 3-50 St. Nicholas Avenue (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-05T20:37:47Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hakimian Capital buys $15.3M note secured by Flushing office building</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/hakimian-capital-buys-15-3m-note-secured-by-flushing-office-building/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hakimian Capital through the entity Horace Harding HC LLC, bought a note with an original</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 163-03 Horace Harding Expressway (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Daryl Hagler, CDK Capital sign $65.8M acquisition loan with Valley for under-construction project in in Ridgewood</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/daryl-hagler-cdk-capital-sign-65-8m-acquisition-loan-with-valley-for-under-construction-project-in-in-ridgewood/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Daryl Hagler and CDK Capital through the entity CDK 3-50 St. Nicholas LLC as borrower</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 3-50 St. Nicholas Avenue (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-06T18:19:10Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hakimian Capital buys $15.3M note secured by Flushing office building</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/hakimian-capital-buys-15-3m-note-secured-by-flushing-office-building/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hakimian Capital through the entity Horace Harding HC LLC, bought a note with an original</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 163-03 Horace Harding Expressway (Credit - Cyclomedia) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Daryl Hagler, CDK Capital sign $65.8M acquisition loan with Valley for under-construction project in in Ridgewood</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/daryl-hagler-cdk-capital-sign-65-8m-acquisition-loan-with-valley-for-under-construction-project-in-in-ridgewood/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Daryl Hagler and CDK Capital through the entity CDK 3-50 St. Nicholas LLC as borrower</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 3-50 St. Nicholas Avenue (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-10T17:19:17Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>$7M internal transfer at Harmony Group medical building in Rockaway Beach</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/7m-internal-transfer-at-harmony-group-medical-building-in-rockaway-beach/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Two entities in care of Uri Kaufman’s Harmony Group Capital sold a stake in the</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 90-01 Beach Channel Drive (Credit - Cyclomedia) Two entities in care of Uri Kaufman’s Harmony Group Capital sold a stake in the medical office building (O7) at 90-01 Beach Channel Drive in Rockaway Beach, Queens, valued at $7 million. In the transfer, Jacqueline Cohen through the entity Nu Trust acquired an interest from Eliahu Kaufman through the entity Mohawk Trust. This building is the historic Rockaway Courthouse. The deal closed on September 28, 2026 and was recorded on October 8, 2026. The property has 35,977 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $194 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In 2022, City Reporter reported that the city’s Economic Development Corporation voted to alter a deed restriction limiting use of the property to medical. Property documents from 2018 show the parcel was subject to a 20-year deed restriction, tied to Uri Kaufman’s acquisition of the property in 2015 for just $50,000. “… for a period of twenty (20) years from the </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Weiss Realty pays $7.2M for two rentals with 103 units in Pelham Bay</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/weiss-realty-pays-7-2m-for-two-rentals-with-103-units-in-pelham-bay/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Weiss Realty through the entity Saint Theresa LLC paid $7.2 million to the entity 2900</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers 2916 St Theresa Avenue (Credit - Cyclomedia) Weiss Realty through the entity Saint Theresa LLC paid $7.2 million to the entity 2900 St Theresa LLC for the 54-unit residential elevator building (D1) at 2900 St Theresa Avenue in Pelham Bay, Bronx and 49-unit residential elevator building (D1) at 2916 St Theresa Avenue in Pelham Bay, Bronx. The expected use is cash flowing. The deal closed on October 7, 2026 and was recorded on October 8, 2026. The two properties have 99,257 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $73 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Evan Schwartz was Evan Schwartz. The signatory for Weiss Realty was Kenneth Yustman . The contract date was August 21, 2026. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is the property on 2916 St Theresa Avenue. Prior sales, articles and revenue Prior to this transaction, Pincu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-11T17:40:27Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,74 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>$7M internal transfer at Harmony Group medical building in Rockaway Beach</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/7m-internal-transfer-at-harmony-group-medical-building-in-rockaway-beach/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Two entities in care of Uri Kaufman’s Harmony Group Capital sold a stake in the</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 90-01 Beach Channel Drive (Credit - Cyclomedia) Two entities in care of Uri Kaufman’s Harmony Group Capital sold a stake in the medical office building (O7) at 90-01 Beach Channel Drive in Rockaway Beach, Queens, valued at $7 million. In the transfer, Jacqueline Cohen through the entity Nu Trust acquired an interest from Eliahu Kaufman through the entity Mohawk Trust. This building is the historic Rockaway Courthouse. The deal closed on September 28, 2026 and was recorded on October 8, 2026. The property has 35,977 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $194 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) In 2022, City Reporter reported that the city’s Economic Development Corporation voted to alter a deed restriction limiting use of the property to medical. Property documents from 2018 show the parcel was subject to a 20-year deed restriction, tied to Uri Kaufman’s acquisition of the property in 2015 for just $50,000. “… for a period of twenty (20) years from the </t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Weiss Realty pays $7.2M for two rentals with 103 units in Pelham Bay</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/weiss-realty-pays-7-2m-for-two-rentals-with-103-units-in-pelham-bay/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Weiss Realty through the entity Saint Theresa LLC paid $7.2 million to the entity 2900</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 2916 St Theresa Avenue (Credit - Cyclomedia) Weiss Realty through the entity Saint Theresa LLC paid $7.2 million to the entity 2900 St Theresa LLC for the 54-unit residential elevator building (D1) at 2900 St Theresa Avenue in Pelham Bay, Bronx and 49-unit residential elevator building (D1) at 2916 St Theresa Avenue in Pelham Bay, Bronx. The expected use is cash flowing. The deal closed on October 7, 2026 and was recorded on October 8, 2026. The two properties have 99,257 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $73 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Evan Schwartz was Evan Schwartz. The signatory for Weiss Realty was Kenneth Yustman . The contract date was August 21, 2026. Because multiple properties have been transacted, some of the following sections will follow the property with the largest assessed value, which in this case, is the property on 2916 St Theresa Avenue. Prior sales, articles and revenue Prior to this transaction, Pincu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-12T21:15:08Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Permits Filed for 44-61 21st Street in Long Island City, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/10/permits-filed-for-44-61-21st-street-in-long-island-city-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Permits have been filed for a 15-story mixed-use building at 44-61 21st Street in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Located at the corner of 44th Drive, the lot is one block from the Court Square–23rd Street station, served by the 7, E, and F trains. Zev Mayer of Walton Developers is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-12T10:30:56+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mon, 12 Oct 2026 10:30:56 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Long Island City</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Vanessa Londono 6:30 am on October 12, 2026 Permits have been filed for a 15-story mixed-use building at 44-61 21st Street in Long Island City, Queens. Located at the corner of 44th Drive, the lot is one block from the Court Square–23rd Street station, served by the 7, E, and F trains. Zev Mayer of Walton Developers is listed as the owner behind the applications. The proposed 165-foot-tall development will yield 108,308 square feet, with 79,778 square feet designated for residential space and 28,530 square feet for commercial space. The building will have 94 residences, most likely rentals based on the average unit scope of 848 square feet. The concrete-based structure will also have a cellar and four enclosed parking spaces. Kao Hwa Lee Architects is listed as the architect of record. Demolition permits were filed last month for the one-story building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-13T19:13:34Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 44-61 21st Street in Long Island City, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/10/permits-filed-for-44-61-21st-street-in-long-island-city-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a 15-story mixed-use building at 44-61 21st Street in &lt;a href="https://newyorkyimby.com/neighborhoods/long-island-city"&gt;Long Island City&lt;/a&gt;, Queens. Located at the corner of 44th Drive, the lot is one block from the Court Square–23rd Street station, served by the 7, E, and F trains. Zev Mayer of Walton Developers is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-12T10:30:56+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Mon, 12 Oct 2026 10:30:56 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Long Island City</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on October 12, 2026 Permits have been filed for a 15-story mixed-use building at 44-61 21st Street in Long Island City, Queens. Located at the corner of 44th Drive, the lot is one block from the Court Square–23rd Street station, served by the 7, E, and F trains. Zev Mayer of Walton Developers is listed as the owner behind the applications. The proposed 165-foot-tall development will yield 108,308 square feet, with 79,778 square feet designated for residential space and 28,530 square feet for commercial space. The building will have 94 residences, most likely rentals based on the average unit scope of 848 square feet. The concrete-based structure will also have a cellar and four enclosed parking spaces. Kao Hwa Lee Architects is listed as the architect of record. Demolition permits were filed last month for the one-story building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-14T17:06:17Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gjovan Rroku files plans for 10 units in Wakefield</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/gjovan-rroku-files-plans-for-10-units-in-wakefield/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gjovan Rroku submitted a new building construction project for a 10-unit, 8,296-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Development 4632 Bronx Boulevard axonometric diagram (Credit - John Backos architect via DOB) Gjovan Rroku submitted a new building construction project for a 10-unit, 8,296-square-foot residential (R-2) building at 4632 Bronx Boulevard in Wakefield, Bronx. The plan was filed on October 12, 2026. It calls for the construction of a 30-foot-tall, three-story building and was filed with the New York City Department of Buildings under job number X01464030. Gjovan Rroku has filed 4 new building projects with 101 new units and 68,564 square feet over the past three years. The project is described in the filing as: new 3-story residential building.. The applicant is the Registered Architect John Backos of Grid Drafting And Consulting . John Backos has filed 50 new building projects with 1,143 new units and 708,756 square feet over the past three years. 4632 Bronx Boulevard The neighborhood In Wakefield, The bulk, or 34 percent of the 9.5 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 27 percent of the space. In sales, Wakefield has near average sales volume among other neighborhoods with $83.3 million in sales volume in the last </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-15T16:55:05Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Gjovan Rroku files plans for 10 units in Wakefield</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/gjovan-rroku-files-plans-for-10-units-in-wakefield/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Gjovan Rroku submitted a new building construction project for a 10-unit, 8,296-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Development 4632 Bronx Boulevard axonometric diagram (Credit - John Backos architect via DOB) Gjovan Rroku submitted a new building construction project for a 10-unit, 8,296-square-foot residential (R-2) building at 4632 Bronx Boulevard in Wakefield, Bronx. The plan was filed on October 12, 2026. It calls for the construction of a 30-foot-tall, three-story building and was filed with the New York City Department of Buildings under job number X01464030. Gjovan Rroku has filed 4 new building projects with 101 new units and 68,564 square feet over the past three years. The project is described in the filing as: new 3-story residential building.. The applicant is the Registered Architect John Backos of Grid Drafting And Consulting . John Backos has filed 50 new building projects with 1,143 new units and 708,756 square feet over the past three years. 4632 Bronx Boulevard The neighborhood In Wakefield, The bulk, or 34 percent of the 9.5 million square feet of commercial built space are walkup buildings, with elevator buildings next occupying 27 percent of the space. In sales, Wakefield has near average sales volume among other neighborhoods with $83.3 million in sales volume in the last </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-16T16:34:12Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T&amp;E Development files plans for 76 units in Chelsea</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/te-development-files-plans-for-76-units-in-chelsea/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>T&amp;E Development , led by Einav Gelberg and Tomer Erlich , submitted a new building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 540 West 29th Street elevation (l.) and axonometric diagram (r.) (Credit - Robert Bianchini architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-17T15:29:15Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>T&amp;E Development files plans for 76 units in Chelsea</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/te-development-files-plans-for-76-units-in-chelsea/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>T&amp;E Development , led by Einav Gelberg and Tomer Erlich , submitted a new building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 540 West 29th Street elevation (l.) and axonometric diagram (r.) (Credit - Robert Bianchini architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-19T18:41:56Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,86 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Seven New Residential Projects Underway in Astoria, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/10/seven-new-residential-projects-underway-in-astoria-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>YIMBY checked in on seven new residential developments underway in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. The projects will add hundreds of new housing units to the southern end of the neighborhood along and below 35th Avenue.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-19T11:00:32+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mon, 19 Oct 2026 11:00:32 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Astoria</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 7:00 am on October 19, 2026 YIMBY checked in on seven new residential developments underway in Astoria, Queens. The projects will add hundreds of new housing units to the southern end of the neighborhood along and below 35th Avenue. Excavation and pilings are progressing at 36-31 31st Street, the site of a nine-story residential building between 36th and 37th Avenues. Completion is slated for next fall, as noted on site. No unit count or architect have been disclosed for the project, and the only DOB zoning diagram shows an outdated iteration from 2015. 36-31 31st Street. Photo by Michael Young. The rendering from the construction board previews a symmetrical design with a setback at the eighth story. The façade will be composed of gray paneling and earth-toned brick surrounding a grid of recessed floor-to-ceiling windows. 36-31 31st Street. Photo by Michael Young.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>South American firm seeks to build approximately 612 apartments in Astoria</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/south-american-firm-seeks-to-build-approximately-612-apartments-in-astoria/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A company affiliated with HC Corporation, a family office based in Uruguay with roots in</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development Approximate boundary of development site, the landmarked property is to the right at 12-12 33rd Avenue Rezoning (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-20T16:57:11Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,66 +473,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Seven New Residential Projects Underway in Astoria, Queens</t>
+          <t>Charles Quimby pays $2.3M to Ralph Giordano for 16-unit walkup in Park Slope</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/10/seven-new-residential-projects-underway-in-astoria-queens.html</t>
+          <t>https://www.pincusco.com/charles-quimby-pays-2-3m-to-ralph-giordano-for-16-unit-walkup-in-park-slope/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>YIMBY checked in on seven new residential developments underway in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. The projects will add hundreds of new housing units to the southern end of the neighborhood along and below 35th Avenue.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-19T11:00:32+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Mon, 19 Oct 2026 11:00:32 +0000</t>
-        </is>
-      </c>
+          <t>Charles A. Quimby through the entity 207 Eighth LLC paid $2.3 million to Ralph Giordano</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>YIMBY</t>
+          <t>PincusCo</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Astoria</t>
+          <t>PincusCo - Home</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Michael Young and Matt Pruznick 7:00 am on October 19, 2026 YIMBY checked in on seven new residential developments underway in Astoria, Queens. The projects will add hundreds of new housing units to the southern end of the neighborhood along and below 35th Avenue. Excavation and pilings are progressing at 36-31 31st Street, the site of a nine-story residential building between 36th and 37th Avenues. Completion is slated for next fall, as noted on site. No unit count or architect have been disclosed for the project, and the only DOB zoning diagram shows an outdated iteration from 2015. 36-31 31st Street. Photo by Michael Young. The rendering from the construction board previews a symmetrical design with a setback at the eighth story. The façade will be composed of gray paneling and earth-toned brick surrounding a grid of recessed floor-to-ceiling windows. 36-31 31st Street. Photo by Michael Young.</t>
+          <t>Transfers 207 8th Avenue (Credit - Cyclomedia) Charles A. Quimby through the entity 207 Eighth LLC paid $2.3 million to Ralph Giordano through the entity 205 207 8th Avenue LLC for the 16-unit residential walkup building (C1) at 207 8th Avenue in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on October 8, 2026 and was recorded on October 16, 2026. The property has 10,444 square feet of built space and 1,748 square feet of additional air rights for a total buildable of 12,201 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $220 and the price per buildable square foot is $188 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ralph Giordano was Ralph Giordano. The signatory for Charles A. Quimby was Charles A. Quimby Jr. . The contract date was June 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Charles A. Quimby purchased one property in one transaction for a total of $4.2 million and has no record i</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>South American firm seeks to build approximately 612 apartments in Astoria</t>
+          <t>Ultimate Care signs $38M refi with Bankwell for industrial in Williamsburg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.pincusco.com/south-american-firm-seeks-to-build-approximately-612-apartments-in-astoria/</t>
+          <t>https://www.pincusco.com/ultimate-care-signs-38m-refi-with-bankwell-for-industrial-in-williamsburg/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A company affiliated with HC Corporation, a family office based in Uruguay with roots in</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
+          <t>Ultimate Care through the entity Kent Ave Property, LLC as borrower signed a refi loan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
@@ -546,7 +534,75 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Development Approximate boundary of development site, the landmarked property is to the right at 12-12 33rd Avenue Rezoning (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+          <t>Transfers 667 Kent Avenue (Credit - Cyclomedia) Ultimate Care through the entity Kent Ave Property, LLC as borrower signed a refi loan with lender Bankwell Bank valued at $38 million for two industrial properties including the industrial building (F5) at 667 Kent Avenue in Williamsburg, Brooklyn and industrial building (F9) at 25 Hooper Street in Williamsburg, Brooklyn. The deal closed on October 9, 2026 and was recorded on October 16, 2026. The prior lender was Bankwell Bank which held debt that had an original loan amount of $32 million. The two properties have 59,597 square feet of built space and 51,384 square feet of additional air rights for a total buildable of 110,956 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $637 and the price per buildable square foot is $342 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ultimate Care was Samuel Gutman and Leopold Friedman . The signatory for Bankwell Bank was Connor Clark . Bankwell Bank has provided $105.5 million through eight</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Stillwater Real Estate pays $3.7M for 10-unit walkup in Brooklyn Heights</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/stillwater-real-estate-pays-3-7m-for-10-unit-walkup-in-brooklyn-heights/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Stillwater Real Estate &amp; Property Group through the entity 87 Joralemon Tic 1 LLC paid</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfers 87 Joralemon Street (Credit - Cyclomedia) Stillwater Real Estate &amp; Property Group through the entity 87 Joralemon Tic 1 LLC paid $3.7 million to Steven Chu through the entity 87 Joralemon LLC for the 10-unit residential walkup building (C1) at 87 Joralemon Street in Brooklyn Heights, Brooklyn. The expected use is cash flowing. The deal closed on October 13, 2026 and was recorded on October 16, 2026. The property has 5,360 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $688 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Steven Chu was Steven Chu. The signatory for Stillwater Real Estate &amp; Property Group was Matthew Bader . The contract date was June 11, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Stillwater Real Estate &amp; Property Group had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Steven Chu had not purchased any other properties </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Related signs $750M refi for approximately 1,700-unit complex in Hell’s Kitchen</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/related-signs-750m-refi-with-wells-fargo-for-approximately-1700-unit-complex-in-hells-kitchen/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Related Companies through the entity Manhattan Plaza, Inc as borrower signed a refi loan with</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Transfers 576 10th Avenue (Credit - Cyclomedia) Related Companies through the entity Manhattan Plaza, Inc as borrower signed a refi loan with lender Wells Fargo valued at $750 million for the 1,689-unit residential elevator building (D6) at 576 10th Avenue in Hell’s Kitchen, Manhattan. The deal closed on September 29, 2026 and was recorded on October 16, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $450 million. The property has 2,099,504 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $357 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Related Companies was Matthew Finkle and David K. Zussman . Wells Fargo has provided $13 billion through 113 loans over the past two years, including $12.3 billion in 99 refi loans, $304.7 million in six acquisition loans, $216.4 million in two new construction loans, $154.3 million in four initial loans, and $85 million in two additional construction loans. The bulk, or 71 percent of the</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-21T17:07:14Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,142 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Charles Quimby pays $2.3M to Ralph Giordano for 16-unit walkup in Park Slope</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/charles-quimby-pays-2-3m-to-ralph-giordano-for-16-unit-walkup-in-park-slope/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Charles A. Quimby through the entity 207 Eighth LLC paid $2.3 million to Ralph Giordano</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Transfers 207 8th Avenue (Credit - Cyclomedia) Charles A. Quimby through the entity 207 Eighth LLC paid $2.3 million to Ralph Giordano through the entity 205 207 8th Avenue LLC for the 16-unit residential walkup building (C1) at 207 8th Avenue in Park Slope, Brooklyn. The expected use is cash flowing. The deal closed on October 8, 2026 and was recorded on October 16, 2026. The property has 10,444 square feet of built space and 1,748 square feet of additional air rights for a total buildable of 12,201 square feet according to a PincusCo analysis of city data. The sale price per built square foot is $220 and the price per buildable square foot is $188 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ralph Giordano was Ralph Giordano. The signatory for Charles A. Quimby was Charles A. Quimby Jr. . The contract date was June 25, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has records that the buyer Charles A. Quimby purchased one property in one transaction for a total of $4.2 million and has no record i</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ultimate Care signs $38M refi with Bankwell for industrial in Williamsburg</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ultimate-care-signs-38m-refi-with-bankwell-for-industrial-in-williamsburg/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Ultimate Care through the entity Kent Ave Property, LLC as borrower signed a refi loan</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Transfers 667 Kent Avenue (Credit - Cyclomedia) Ultimate Care through the entity Kent Ave Property, LLC as borrower signed a refi loan with lender Bankwell Bank valued at $38 million for two industrial properties including the industrial building (F5) at 667 Kent Avenue in Williamsburg, Brooklyn and industrial building (F9) at 25 Hooper Street in Williamsburg, Brooklyn. The deal closed on October 9, 2026 and was recorded on October 16, 2026. The prior lender was Bankwell Bank which held debt that had an original loan amount of $32 million. The two properties have 59,597 square feet of built space and 51,384 square feet of additional air rights for a total buildable of 110,956 square feet according to a PincusCo analysis of city data. The loan price per built square foot is $637 and the price per buildable square foot is $342 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Ultimate Care was Samuel Gutman and Leopold Friedman . The signatory for Bankwell Bank was Connor Clark . Bankwell Bank has provided $105.5 million through eight</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Stillwater Real Estate pays $3.7M for 10-unit walkup in Brooklyn Heights</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/stillwater-real-estate-pays-3-7m-for-10-unit-walkup-in-brooklyn-heights/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Stillwater Real Estate &amp; Property Group through the entity 87 Joralemon Tic 1 LLC paid</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transfers 87 Joralemon Street (Credit - Cyclomedia) Stillwater Real Estate &amp; Property Group through the entity 87 Joralemon Tic 1 LLC paid $3.7 million to Steven Chu through the entity 87 Joralemon LLC for the 10-unit residential walkup building (C1) at 87 Joralemon Street in Brooklyn Heights, Brooklyn. The expected use is cash flowing. The deal closed on October 13, 2026 and was recorded on October 16, 2026. The property has 5,360 square feet of built space according to a PincusCo analysis of city data. The sale price per built square foot is $688 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Steven Chu was Steven Chu. The signatory for Stillwater Real Estate &amp; Property Group was Matthew Bader . The contract date was June 11, 2026. Prior sales, articles and revenue Prior to this transaction, PincusCo has no record that the buyer Stillwater Real Estate &amp; Property Group had purchased any other properties and has no record it sold any properties over the past 24 months. The seller Steven Chu had not purchased any other properties </t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Related signs $750M refi for approximately 1,700-unit complex in Hell’s Kitchen</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/related-signs-750m-refi-with-wells-fargo-for-approximately-1700-unit-complex-in-hells-kitchen/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Related Companies through the entity Manhattan Plaza, Inc as borrower signed a refi loan with</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Transfers 576 10th Avenue (Credit - Cyclomedia) Related Companies through the entity Manhattan Plaza, Inc as borrower signed a refi loan with lender Wells Fargo valued at $750 million for the 1,689-unit residential elevator building (D6) at 576 10th Avenue in Hell’s Kitchen, Manhattan. The deal closed on September 29, 2026 and was recorded on October 16, 2026. The prior lender was Fannie Mae which held debt that had an original loan amount of $450 million. The property has 2,099,504 square feet of built space according to a PincusCo analysis of city data. The loan price per built square foot is $357 per the PincusCo analysis. (The price per square foot analysis is the transaction price divided by square feet as reported in public records and assumes no air rights have been sold.) The signatory for Related Companies was Matthew Finkle and David K. Zussman . Wells Fargo has provided $13 billion through 113 loans over the past two years, including $12.3 billion in 99 refi loans, $304.7 million in six acquisition loans, $216.4 million in two new construction loans, $154.3 million in four initial loans, and $85 million in two additional construction loans. The bulk, or 71 percent of the</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-22T17:06:49Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,48 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>560-Unit Tower Readies for Groundbreaking at 35-10 Steinway Street in Astoria, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/10/560-unit-tower-readies-for-groundbreaking-at-35-10-steinway-street-in-astoria-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Demolition is complete at 35-10 Steinway Street, the site of a 27-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Designed by Beyer Blinder Belle and developed in a joint venture between LMXD and BedRock Real Estate Partners, the nearly 500,000-square-foot structure will yield 560 rental units in studio to three-bedroom layouts. The all-electric project will also include ground-floor retail space for P.C. Richard &amp;#38; Son. The property is bounded by 35th Avenue to the northeast, 38th Street to the northwest, and Steinway Street to the southeast.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-22T12:00:36+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Thu, 22 Oct 2026 12:00:36 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Astoria</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Michael Young and Matt Pruznick 8:00 am on October 22, 2026 Demolition is complete at 35-10 Steinway Street, the site of a 27-story mixed-use residential building in Astoria, Queens. Designed by Beyer Blinder Belle and developed in a joint venture between LMXD and BedRock Real Estate Partners, the nearly 500,000-square-foot structure will yield 560 rental units in studio to three-bedroom layouts. The all-electric project will also include ground-floor retail space for P.C. Richard &amp; Son. The property is bounded by 35th Avenue to the northeast, 38th Street to the northwest, and Steinway Street to the southeast. The site has been cleared of its former surface-level parking lot, with a lone heap of asphalt rubble remaining. Construction machinery has yet to arrive at the property, but it’s possible that excavation could get underway before the end of the year. 35-10 Steinway Street. Photo by Michael Young. 35-10 Steinway Street. Photo by Michael Young. 35-10 Steinway Street. Photo by Michael Young.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-23T17:01:22Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -473,27 +473,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>560-Unit Tower Readies for Groundbreaking at 35-10 Steinway Street in Astoria, Queens</t>
+          <t>Permits Filed for 41-22 44th Street in Sunnyside, Queens</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://newyorkyimby.com/2026/10/560-unit-tower-readies-for-groundbreaking-at-35-10-steinway-street-in-astoria-queens.html</t>
+          <t>https://newyorkyimby.com/2026/10/permits-filed-for-41-22-44th-street-in-sunnyside-queens.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Demolition is complete at 35-10 Steinway Street, the site of a 27-story mixed-use residential building in &lt;a href="https://newyorkyimby.com/neighborhoods/astoria"&gt;Astoria&lt;/a&gt;, Queens. Designed by Beyer Blinder Belle and developed in a joint venture between LMXD and BedRock Real Estate Partners, the nearly 500,000-square-foot structure will yield 560 rental units in studio to three-bedroom layouts. The all-electric project will also include ground-floor retail space for P.C. Richard &amp;#38; Son. The property is bounded by 35th Avenue to the northeast, 38th Street to the northwest, and Steinway Street to the southeast.</t>
+          <t>Permits have been filed for an eight-story residential building at 41-22 44th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Located between 43rd Avenue and Skillman Avenue, the lot is closest to the 46th Street–Bliss Street subway station, served by the 7 train. Guan Shawn Wang of 5615 Van Cleef Real Estate LLC is listed as the owner behind the applications.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-22T12:00:36+00:00</t>
+          <t>2026-10-23T10:30:48+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 12:00:36 +0000</t>
+          <t>Fri, 23 Oct 2026 10:30:48 +0000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -503,12 +503,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>YIMBY - Astoria</t>
+          <t>YIMBY - Sunnyside</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>By: Michael Young and Matt Pruznick 8:00 am on October 22, 2026 Demolition is complete at 35-10 Steinway Street, the site of a 27-story mixed-use residential building in Astoria, Queens. Designed by Beyer Blinder Belle and developed in a joint venture between LMXD and BedRock Real Estate Partners, the nearly 500,000-square-foot structure will yield 560 rental units in studio to three-bedroom layouts. The all-electric project will also include ground-floor retail space for P.C. Richard &amp; Son. The property is bounded by 35th Avenue to the northeast, 38th Street to the northwest, and Steinway Street to the southeast. The site has been cleared of its former surface-level parking lot, with a lone heap of asphalt rubble remaining. Construction machinery has yet to arrive at the property, but it’s possible that excavation could get underway before the end of the year. 35-10 Steinway Street. Photo by Michael Young. 35-10 Steinway Street. Photo by Michael Young. 35-10 Steinway Street. Photo by Michael Young.</t>
+          <t>By: Vanessa Londono 6:30 am on October 23, 2026 Permits have been filed for an eight-story residential building at 41-22 44th Street in Sunnyside, Queens. Located between 43rd Avenue and Skillman Avenue, the lot is closest to the 46th Street–Bliss Street subway station, served by the 7 train. Guan Shawn Wang of 5615 Van Cleef Real Estate LLC is listed as the owner behind the applications. The proposed 83-foot-tall development will yield 19,981 square feet designated for residential space. The building will have 29 residences, most likely rentals based on the average unit scope of 689 square feet. The concrete-based structure will also have a cellar, an eighth-floor roof terrace, and a 31-foot-long rear yard. Murat Mutlu of INOA Architecture Inc. is listed as the architect of record. Demolition permits were filed in April for the two-story residential building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-24T15:52:31Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,48 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 41-22 44th Street in Sunnyside, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/10/permits-filed-for-41-22-44th-street-in-sunnyside-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for an eight-story residential building at 41-22 44th Street in &lt;a href="https://newyorkyimby.com/neighborhoods/sunnyside"&gt;Sunnyside&lt;/a&gt;, Queens. Located between 43rd Avenue and Skillman Avenue, the lot is closest to the 46th Street–Bliss Street subway station, served by the 7 train. Guan Shawn Wang of 5615 Van Cleef Real Estate LLC is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-23T10:30:48+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Fri, 23 Oct 2026 10:30:48 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Sunnyside</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on October 23, 2026 Permits have been filed for an eight-story residential building at 41-22 44th Street in Sunnyside, Queens. Located between 43rd Avenue and Skillman Avenue, the lot is closest to the 46th Street–Bliss Street subway station, served by the 7 train. Guan Shawn Wang of 5615 Van Cleef Real Estate LLC is listed as the owner behind the applications. The proposed 83-foot-tall development will yield 19,981 square feet designated for residential space. The building will have 29 residences, most likely rentals based on the average unit scope of 689 square feet. The concrete-based structure will also have a cellar, an eighth-floor roof terrace, and a 31-foot-long rear yard. Murat Mutlu of INOA Architecture Inc. is listed as the architect of record. Demolition permits were filed in April for the two-story residential building on the site. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-26T18:39:28Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,86 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Permits Filed for 161-05 Hillside Avenue in Jamaica, Queens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://newyorkyimby.com/2026/10/permits-filed-for-161-05-hillside-avenue-in-jamaica-queens.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Permits have been filed for a 14-story mixed-use building at 161-05 Hillside Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/jamaica"&gt;Jamaica&lt;/a&gt;, Queens. Located between 161st Street and 162nd Street, the lot is near the Parsons Boulevard subway station, served by the E and F trains. Sandi Silk of Mural Real Estate Partners is listed as the owner behind the applications.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-26T10:30:26+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Mon, 26 Oct 2026 10:30:26 +0000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>YIMBY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>YIMBY - Jamaica</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>By: Vanessa Londono 6:30 am on October 26, 2026 Permits have been filed for a 14-story mixed-use building at 161-05 Hillside Avenue in Jamaica, Queens. Located between 161st Street and 162nd Street, the lot is near the Parsons Boulevard subway station, served by the E and F trains. Sandi Silk of Mural Real Estate Partners is listed as the owner behind the applications. The proposed 144-foot-tall development will yield 125,484 square feet, with 116,061 square feet designated for residential space and 9,422 square feet for commercial space. The building will have 173 residences, most likely rentals based on the average unit scope of 670 square feet. The concrete-based structure will also have a cellar and a 30-foot-long rear yard. Curtis+Ginsberg Architects is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ZD Jasper Realty files plans for 93 units in Astoria, second at two-tower complex</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/zd-jasper-realty-files-plans-for-93-units-in-astoria-second-at-two-tower-complex/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ZD Jasper Realty submitted a new building construction project for a 93-unit, 91,240-square-foot residential (R-2)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NaT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Development Top Story 35-24 41st Street (l.) and 35-25 Steinway Street (r.) axonometric diagrams (Credit - Jeremiah Zuidema architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-27T17:57:23Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,86 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Permits Filed for 161-05 Hillside Avenue in Jamaica, Queens</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://newyorkyimby.com/2026/10/permits-filed-for-161-05-hillside-avenue-in-jamaica-queens.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Permits have been filed for a 14-story mixed-use building at 161-05 Hillside Avenue in &lt;a href="https://newyorkyimby.com/neighborhoods/jamaica"&gt;Jamaica&lt;/a&gt;, Queens. Located between 161st Street and 162nd Street, the lot is near the Parsons Boulevard subway station, served by the E and F trains. Sandi Silk of Mural Real Estate Partners is listed as the owner behind the applications.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-10-26T10:30:26+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Mon, 26 Oct 2026 10:30:26 +0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>YIMBY</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>YIMBY - Jamaica</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>By: Vanessa Londono 6:30 am on October 26, 2026 Permits have been filed for a 14-story mixed-use building at 161-05 Hillside Avenue in Jamaica, Queens. Located between 161st Street and 162nd Street, the lot is near the Parsons Boulevard subway station, served by the E and F trains. Sandi Silk of Mural Real Estate Partners is listed as the owner behind the applications. The proposed 144-foot-tall development will yield 125,484 square feet, with 116,061 square feet designated for residential space and 9,422 square feet for commercial space. The building will have 173 residences, most likely rentals based on the average unit scope of 670 square feet. The concrete-based structure will also have a cellar and a 30-foot-long rear yard. Curtis+Ginsberg Architects is listed as the architect of record. Demolition permits have not been filed yet. An estimated completion date has not been announced. Subscribe to YIMBY’s daily e-mail Follow YIMBYgram for real-time photo updates Like YIMBY on Facebook Follow YIMBY’s Twitter for the latest in YIMBYnews</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ZD Jasper Realty files plans for 93 units in Astoria, second at two-tower complex</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/zd-jasper-realty-files-plans-for-93-units-in-astoria-second-at-two-tower-complex/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ZD Jasper Realty submitted a new building construction project for a 93-unit, 91,240-square-foot residential (R-2)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NaT</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Development Top Story 35-24 41st Street (l.) and 35-25 Steinway Street (r.) axonometric diagrams (Credit - Jeremiah Zuidema architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-28T18:19:45Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,40 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ben Kaftari files plans for 56 units in Briarwood</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/ben-kaftari-files-plans-for-56-units-in-briarwood/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ben Kaftari submitted a new building construction project for a 56-unit, 54,052-square-foot residential (R-2) building</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Development 139-57 Queens Boulevard axonometric diagram (Credit - Naresh Mahangu professional engineer via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-29T18:25:36Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,40 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ben Kaftari files plans for 56 units in Briarwood</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.pincusco.com/ben-kaftari-files-plans-for-56-units-in-briarwood/</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Ben Kaftari submitted a new building construction project for a 56-unit, 54,052-square-foot residential (R-2) building</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PincusCo</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PincusCo - Home</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Development 139-57 Queens Boulevard axonometric diagram (Credit - Naresh Mahangu professional engineer via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto update queens news 2026-10-30T17:59:00Z
</commit_message>
<xml_diff>
--- a/data/output/queens_dev_news.xlsx
+++ b/data/output/queens_dev_news.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,74 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>content_preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CAVU Property signs $72.6M construction loan for two LIC projects with 174 units total</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/cavu-property-signs-72-6m-construction-loan-for-two-lic-projects-with-174-units-total/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CAVU Property Group through the entity LIC Bldg 32 LLC as borrower signed a new</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Transfers 38-11 32nd Street (l.) and 38-12 33rd Street (r.) axonometric diagrams (Credit - Joseph Frankl architect via DOB) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Big Six Towers co-op in Woodside signs $141.9M rehab construction loan with city</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.pincusco.com/big-six-towers-co-op-in-woodside-signs-141-9m-rehab-construction-loan-with-city/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Big Six Towers Cooperative through the entity Big Six Towers, Inc. as borrower signed a</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PincusCo</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PincusCo - Home</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Transfers Bix Six Towers cooperative (Credit - Google Earth) Continue reading with a PincusCo subscription Sign up for a paid subscription to view this content. Already a subscriber? Log in here. Continue Reading</t>
         </is>
       </c>
     </row>

</xml_diff>